<commit_message>
PAUSED (task118): architecture 2 green at stage 5 and judged DETERMINISTIC on pass 7, the corrections ask's device moved from the autosaves (filed in 7.3) to schedules set back to draft; guard heart BLOCKs on ban.strategy and ban.pattern against task139 v2, the author's ban waiver owed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Es2YJxT597uNAuNJZNdYR4
</commit_message>
<xml_diff>
--- a/task118/golden/squad_placement_2027.xlsx
+++ b/task118/golden/squad_placement_2027.xlsx
@@ -9,18 +9,19 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desks" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Click chain" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back-test" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pages" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Back-test" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Desks'!$A$4:$E$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Desks'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Desks'!$A$1:$E$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Click chain'!$3:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Click chain'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Back-test'!$3:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Back-test'!$A$1:$I$13</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Notes'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Click chain'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Pages'!$3:$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Pages'!$A$1:$E$27</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Back-test'!$3:$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Back-test'!$A$1:$M$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -107,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,7 +132,13 @@
     <xf numFmtId="10" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -140,23 +147,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,9 +523,9 @@
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,7 +538,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Readers, visits and minutes cover October 2025 to September 2026.</t>
+          <t>Corrections: articles first published from October 2025 to September 2026 whose headline was corrected.</t>
         </is>
       </c>
     </row>
@@ -560,17 +555,17 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Average monthly readers</t>
+          <t>Median minutes to first headline correction</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Average monthly visits</t>
+          <t>First corrections within an hour</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Median minutes to first headline correction</t>
+          <t>First corrections after more than three hours</t>
         </is>
       </c>
     </row>
@@ -586,13 +581,13 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>3180000</v>
+        <v>86</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>13041000</v>
+        <v>14</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>86</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -607,34 +602,34 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>470000</v>
+        <v>55</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1550000</v>
+        <v>9</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Business·national</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>BUS-N</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>1760000</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>6642000</v>
-      </c>
-      <c r="E7" s="6" t="n">
+      <c r="C7" s="9" t="n">
         <v>89</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -649,13 +644,13 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2931000</v>
+        <v>47</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>11626000</v>
+        <v>23</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -670,47 +665,47 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>617000</v>
+        <v>102</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>2359000</v>
+        <v>12</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>102</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Culture·national</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>CUL-N</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
-        <v>1412000</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>5052000</v>
-      </c>
-      <c r="E10" s="9" t="n">
+      <c r="C10" s="6" t="n">
         <v>119</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Recommended: Culture·national, 1,250,000 extra article clicks in 2027. Runner-up Local·metro, 450,000 behind.</t>
+          <t>Recommended: Business·national, 500,000 extra article clicks in 2027. Runner-up Local·metro, 100,000 behind.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Extra clicks for every desk are on the Click chain sheet. Readers and visits to the nearest thousand; definitions on the Notes sheet.</t>
+          <t>Extra clicks for every desk are on the Click chain sheet.</t>
         </is>
       </c>
     </row>
@@ -727,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -737,12 +732,14 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>From each desk's 2027 clicks to the clicks the squad adds</t>
+          <t>From each desk's 2027 clicks to the clicks the squad adds to Bightline</t>
         </is>
       </c>
     </row>
@@ -759,7 +756,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Clicks from Bightline surfaces</t>
+          <t>From Bightline's own pages</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -778,6 +775,16 @@
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Clicks the winning headlines win</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Share new to Bightline</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Extra article clicks 2027</t>
         </is>
@@ -786,26 +793,32 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Culture·national</t>
+          <t>Business·national</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>153350000</v>
+        <v>309100000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>76900000</v>
+        <v>86350000</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>6600000</v>
+        <v>51450000</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>70300000</v>
+        <v>34900000</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0.01780987549676022</v>
+        <v>0.01999385765112825</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>1250000</v>
+        <v>700000</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>0.7111513837918686</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>500000</v>
       </c>
     </row>
     <row r="5">
@@ -826,36 +839,48 @@
       <c r="E5" s="6" t="n">
         <v>31450000</v>
       </c>
-      <c r="F5" s="13" t="n">
-        <v>0.02569565737860459</v>
+      <c r="F5" s="14" t="n">
+        <v>0.02569565727821913</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>800000</v>
       </c>
+      <c r="H5" s="15" t="n">
+        <v>0.4856660312302004</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>400000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Business·national</t>
+          <t>Culture·national</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>309050000</v>
+        <v>153350000</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>86350000</v>
+        <v>76900000</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>51450000</v>
+        <v>6600000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>34900000</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0.01999385769563704</v>
+        <v>70300000</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>0.01780987544338385</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>700000</v>
+        <v>1250000</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>0.2686263827208286</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>350000</v>
       </c>
     </row>
     <row r="7">
@@ -865,7 +890,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>341000000</v>
+        <v>340950000</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>98200000</v>
@@ -876,12 +901,18 @@
       <c r="E7" s="6" t="n">
         <v>49050000</v>
       </c>
-      <c r="F7" s="13" t="n">
-        <v>0.01321402065171128</v>
+      <c r="F7" s="14" t="n">
+        <v>0.01321402062157698</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>650000</v>
       </c>
+      <c r="H7" s="15" t="n">
+        <v>0.500914766936855</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>300000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -890,7 +921,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>376250000</v>
+        <v>376300000</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>71400000</v>
@@ -901,12 +932,18 @@
       <c r="E8" s="6" t="n">
         <v>43200000</v>
       </c>
-      <c r="F8" s="13" t="n">
-        <v>0.01279192116089391</v>
+      <c r="F8" s="14" t="n">
+        <v>0.01279192113836527</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>550000</v>
       </c>
+      <c r="H8" s="15" t="n">
+        <v>0.5750052627380324</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>300000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -926,31 +963,44 @@
       <c r="E9" s="6" t="n">
         <v>25500000</v>
       </c>
-      <c r="F9" s="13" t="n">
-        <v>0.003937840024793244</v>
+      <c r="F9" s="14" t="n">
+        <v>0.003937839899962059</v>
       </c>
       <c r="G9" s="6" t="n">
         <v>100000</v>
       </c>
+      <c r="H9" s="15" t="n">
+        <v>0.4694175240841066</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>50000</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Bightline surfaces: web home, web section fronts, app home feed, app section tabs and related links. Search, Discover, partner apps, social, newsletters and alerts show the headline stored at publication.</t>
+          <t>Bightline's own pages: the web home pages and section fronts, the app home feed and tabs, and the related-story links on article pages. Search, Discover-style cards, partner apps, social cards, newsletters and alerts keep the headline stored at publication.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>A desk's own tests ship their winners inside the clicks the plan carries forward, so the squad's gain is counted only on headlines the desk does not already test.</t>
+          <t>The squad takes the headlines a desk has not put under test itself; a desk's own winners already ship inside the clicks the plan carries forward.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Extra clicks = shrunk winning lift x clicks on headlines the desk does not test, on unrounded clicks. Click columns rounded to the nearest 50,000.</t>
+          <t>A winning headline's extra clicks on a page are new to Bightline only in the share of that page's views that would otherwise end with no article click (one minus the page's click-through, Pages sheet); the rest are clicks the headlines beside it lose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Extra clicks = shrunk winning lift x each page's untested clicks x (1 - that page's click-through), on unrounded clicks. Click columns rounded to the nearest 50,000.</t>
         </is>
       </c>
     </row>
@@ -966,321 +1016,472 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The method against the squad's seven finished embeddings</t>
+          <t>Page click-through, October 2025 to September 2026</t>
         </is>
       </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Embedding</t>
+          <t>Page</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Desk</t>
+          <t>Page views</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>Article click-throughs</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Tests</t>
+          <t>Click-through</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Observed winning lift</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Shrunk winning lift</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Realised holdback lift</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Prediction against realised</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Within 2%</t>
+          <t>Share of views new clicks can come from</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>2019</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <v>72</v>
-      </c>
-      <c r="E4" s="16" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F4" s="13" t="n">
-        <v>0.01863421530172949</v>
-      </c>
-      <c r="G4" s="13" t="n">
-        <v>0.01842</v>
-      </c>
-      <c r="H4" s="17" t="n">
-        <v>0.01162949520789813</v>
-      </c>
-      <c r="I4" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>187485281</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>80855995</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>0.4312658282758741</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>0.5687341717241259</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Wellness</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>2020</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>54</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>0.01440910886894175</v>
-      </c>
-      <c r="G5" s="13" t="n">
-        <v>0.01426</v>
-      </c>
-      <c r="H5" s="17" t="n">
-        <v>0.01045644242228216</v>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/brisbane/</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>152596070</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>71738385</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>0.4701194794859396</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>0.5298805205140604</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Puzzles</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>0.02222330089628922</v>
-      </c>
-      <c r="G6" s="13" t="n">
-        <v>0.02218</v>
-      </c>
-      <c r="H6" s="17" t="n">
-        <v>0.001952249607268808</v>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/brisbane/local/</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>42381145</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>29164383</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>0.6881452353399136</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>0.3118547646600864</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>Recipes</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>88</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>0.037</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>0.02567696027189502</v>
-      </c>
-      <c r="G7" s="13" t="n">
-        <v>0.02554</v>
-      </c>
-      <c r="H7" s="17" t="n">
-        <v>0.005362579165819392</v>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/brisbane/politics/</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>11534448</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>7389518</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>0.6406477362419077</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0.3593522637580923</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Games</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>66</v>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>0.006931499157418917</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <v>0.00695</v>
-      </c>
-      <c r="H8" s="17" t="n">
-        <v>-0.002661991738285296</v>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/brisbane/sport/</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>19186394</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>14407546</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>0.7509251608196934</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>0.2490748391803066</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>Recipes</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <v>0.0110064402337643</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>0.01108</v>
-      </c>
-      <c r="H9" s="17" t="n">
-        <v>-0.006638968071813967</v>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/business/</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>9867412</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>6221630</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>0.6305229780615221</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0.3694770219384779</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Wellness</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>2025</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>58</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>0.032</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>0.02410076612859266</v>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>0.02431</v>
-      </c>
-      <c r="H10" s="17" t="n">
-        <v>-0.008606905446620572</v>
-      </c>
-      <c r="I10" s="18" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/culture/</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>46013257</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>38259637</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>0.8314916068645173</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.1685083931354827</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Within 2%</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr">
-        <is>
-          <t>7 of 7</t>
-        </is>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/politics/</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>14860121</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>9837950</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>0.6620370049476717</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>0.3379629950523283</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>bightline.com.au/sport/</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>29657913</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>21415938</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>0.7220986183350123</v>
+      </c>
+      <c r="E12" s="15" t="n">
+        <v>0.2779013816649877</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Prediction = the shrunk winning lift of the embedding's tests; realised = the change log's lift over the 5 per cent holdback for the year.</t>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Home feed</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>494832604</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>202744444</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>0.4097232930108219</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>0.5902767069891781</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Related stories (article pages)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>900056801</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>108153068</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>0.1201624918336682</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.8798375081663319</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Brisbane Local</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>11318758</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>7595566</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>0.6710600226632639</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>0.3289399773367361</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Brisbane Politics</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>4807407</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>2988363</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>0.6216163932032382</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0.3783836067967618</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Brisbane Sport</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>8390566</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>6142547</v>
+      </c>
+      <c r="D17" s="15" t="n">
+        <v>0.7320777883160683</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>0.2679222116839317</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Business</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>6946510</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>4310363</v>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>0.6205077081872767</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0.3794922918127233</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Culture</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>28732821</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>23292380</v>
+      </c>
+      <c r="D19" s="15" t="n">
+        <v>0.8106541296449798</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>0.1893458703550202</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Games</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>11004565</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>8126966</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>0.738508609836009</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0.261491390163991</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Politics</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>6873722</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>4396755</v>
+      </c>
+      <c r="D21" s="15" t="n">
+        <v>0.639646904544583</v>
+      </c>
+      <c r="E21" s="15" t="n">
+        <v>0.360353095455417</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Puzzles</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>41315166</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>33109541</v>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>0.8013895188028531</v>
+      </c>
+      <c r="E22" s="15" t="n">
+        <v>0.1986104811971469</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Recipes</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>10341636</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>6822623</v>
+      </c>
+      <c r="D23" s="15" t="n">
+        <v>0.6597237613081721</v>
+      </c>
+      <c r="E23" s="15" t="n">
+        <v>0.3402762386918279</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Sport</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>14143712</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>9897806</v>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>0.6998025695093339</v>
+      </c>
+      <c r="E24" s="15" t="n">
+        <v>0.3001974304906661</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Tab: Wellness</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>10725002</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>7615081</v>
+      </c>
+      <c r="D25" s="15" t="n">
+        <v>0.7100307300641995</v>
+      </c>
+      <c r="E25" s="15" t="n">
+        <v>0.2899692699358005</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Click-through = article click-throughs over page views, twelve months summed (page performance export).</t>
         </is>
       </c>
     </row>
@@ -1296,130 +1497,432 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Definitions and sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Prepared</t>
-        </is>
-      </c>
-      <c r="B3" s="21" t="inlineStr">
-        <is>
-          <t>19 October 2026, for the planning meeting on 4 November 2026</t>
+          <t>The method against the squad's seven finished embeddings</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Embedding</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Desk</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Observed winning lift</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Shrunk winning lift</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Realised holdback lift</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Lift: prediction against realised</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Planned clicks</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Share new to Bightline</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Predicted extra clicks</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Extra clicks against holdback</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Clicks: prediction against measured</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
-        <is>
-          <t>Extra article clicks 2027</t>
-        </is>
-      </c>
-      <c r="B4" s="21" t="inlineStr">
-        <is>
-          <t>Clicks the squad would add in the twelve months after it embeds, counted at the owning desk. 2027 clicks are the audience plan's, which holds each desk at October 2025 to September 2026.</t>
-        </is>
+      <c r="A4" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>72</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>0.0186342151917807</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>0.01842</v>
+      </c>
+      <c r="H4" s="18" t="n">
+        <v>0.01162948923890883</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>36436680</v>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>0.5407319049005754</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>362920</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>357677</v>
+      </c>
+      <c r="M4" s="18" t="n">
+        <v>0.014657348907821</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
-        <is>
-          <t>Winning lift</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>Shipped headline's click-through over the control's, minus one; zero when the control is kept (field reference). Shrunk with one normal prior fitted by maximum likelihood on all 10,111 variant packages in the archive; a desk's lift is the mean over its tests.</t>
-        </is>
+      <c r="A5" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Wellness</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>54</v>
+      </c>
+      <c r="E5" s="15" t="n">
+        <v>0.031</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>0.01440910874370718</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>0.01426</v>
+      </c>
+      <c r="H5" s="18" t="n">
+        <v>0.01045643364005433</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>22853516</v>
+      </c>
+      <c r="J5" s="15" t="n">
+        <v>0.5608991406902406</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>182792</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>185020</v>
+      </c>
+      <c r="M5" s="18" t="n">
+        <v>-0.01204162062204905</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>Average monthly readers</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Panel unique audience for the desk's section, mean of October 2025 to September 2026. Releases up to R26-03 are read on the earlier section list; R26-04, the release log's first release on the 2026 content taxonomy, and every release after it, the R26-04H history release included, are read on the 2026 list. A section's figure for a month is the latest release of that month: the history release replaces three national sections for November to February, and R26-07B, the restatement, replaces April to June on both sites. The July file's April to June rows repeat, figure for figure, the releases R26-07B replaced; they are those figures carried again, not a later release of the months.</t>
-        </is>
+      <c r="A6" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Puzzles</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>0.0222233008182623</v>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>0.02218</v>
+      </c>
+      <c r="H6" s="18" t="n">
+        <v>0.001952246089373499</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>47950584</v>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>0.359025223080722</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>381839</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>386958</v>
+      </c>
+      <c r="M6" s="18" t="n">
+        <v>-0.01322855445536464</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
-        <is>
-          <t>Average monthly visits</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Panel visits for the same section and months, from the same releases.</t>
-        </is>
+      <c r="A7" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Recipes</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>88</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.0256769601553108</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0.02554</v>
+      </c>
+      <c r="H7" s="18" t="n">
+        <v>0.005362574601049719</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>41413944</v>
+      </c>
+      <c r="J7" s="15" t="n">
+        <v>0.7046919437754708</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>745361</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>745627</v>
+      </c>
+      <c r="M7" s="18" t="n">
+        <v>-0.0003564561429945101</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Headline corrections</t>
-        </is>
-      </c>
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>A new correction note on a version readers saw, where a corrected headline went up with it: on the same version, or, where the fix and the note went on separate saves (at most ten minutes apart, CMS export field notes), on a version within those ten minutes before or after it that changed the headline with no new note of its own. A live blog's note is matched to the entry whose headline changed within the ten minutes (editorial standards 7.4 and 7.5). The correction is counted once, on the version that published the headline. Versions readers saw are live saves and a scheduled version the CMS published; drafts are not published. Notes carry forward on later saves and are not counted again, nor is a note put back after a save that left it off; every other new note is a correction to text.</t>
-        </is>
+      <c r="A8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>66</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>0.006931499068715015</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>0.00695</v>
+      </c>
+      <c r="H8" s="18" t="n">
+        <v>-0.00266200450143661</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>39321251</v>
+      </c>
+      <c r="J8" s="15" t="n">
+        <v>0.5407319049005754</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>147773</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>148729</v>
+      </c>
+      <c r="M8" s="18" t="n">
+        <v>-0.006430003924517647</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>Articles</t>
-        </is>
-      </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>Articles first published October 2025 to September 2026 that went live. Live-blog posts, copies restored after the 14 November 2025 Brisbane outage and documents carried across at the 1 October 2025 CMS migration are not separate articles; a restored copy continues its original.</t>
-        </is>
+      <c r="A9" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Recipes</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>0.01100644012240408</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0.01108</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>-0.006638978122375905</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>47851050</v>
+      </c>
+      <c r="J9" s="15" t="n">
+        <v>0.7046919437754708</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>373620</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>376917</v>
+      </c>
+      <c r="M9" s="18" t="n">
+        <v>-0.008746318810068154</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Median minutes</t>
-        </is>
-      </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>Minutes from an article going live to its first headline correction, over corrected articles. An article goes live at its first published version: the time the editor set when the CMS published a scheduled article, otherwise its first live save. The CMS keeps that time on the newsroom's Brisbane clock (AEST, ten hours ahead of the UTC save times); on that clock it falls before the first live save of every article the CMS published. A restored copy keeps its original's time, and an entry's correction counts for its live blog.</t>
-        </is>
+      <c r="A10" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Wellness</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>58</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>0.02410076603605748</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>0.02431</v>
+      </c>
+      <c r="H10" s="18" t="n">
+        <v>-0.008606909253085937</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>27583679</v>
+      </c>
+      <c r="J10" s="15" t="n">
+        <v>0.5608991406902406</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>376116</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>379602</v>
+      </c>
+      <c r="M10" s="18" t="n">
+        <v>-0.009183040318162528</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
-        <is>
-          <t>Sources</t>
-        </is>
-      </c>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>2027 audience plan; pageviews by source and age, Oct 2025 to Sep 2026; headline test archive 2019 to 2026; newsroom staff list; headline squad change log; panel monthly audience and reference workbook; CMS revisions for the web desks and their field notes.</t>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Within 2%</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>7 of 7</t>
+        </is>
+      </c>
+      <c r="M11" s="19" t="inlineStr">
+        <is>
+          <t>7 of 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Lift: the shrunk winning lift of the embedding's tests against the change log's realised lift over the 5 per cent reader holdback. The raw winning lift is within 2% for none of 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Clicks: planned clicks x realised lift x the desk's share new to Bightline (its pages' click-through, weighted by where its clicks start) against the extra clicks measured against the holdback. One share for every embedding, their average 57.0%, is within 2% for 2 of 7 and misses by up to 57%.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>